<commit_message>
Dokuman: tanitim Excel v1.1 — denetim icerigi (UC-28), MUID (UC-29), karsilik beyani (UC-27), GenAI/Agentic kategoriler, PROVISION-IMPACT kurali
</commit_message>
<xml_diff>
--- a/mrm-archer/MRM_Konsolu_Yazilim_Tanitim.xlsx
+++ b/mrm-archer/MRM_Konsolu_Yazilim_Tanitim.xlsx
@@ -19,12 +19,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Menü Envanteri'!$A$3:$F$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'İşlemler (Use-Case)'!$A$3:$H$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Formlar &amp; Alanlar'!$A$3:$F$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'İşlemler (Use-Case)'!$A$3:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Formlar &amp; Alanlar'!$A$3:$F$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Veri Modeli'!$A$3:$D$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roller &amp; Yetki'!$A$3:$F$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hesaplamalar'!$A$3:$C$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bildirim &amp; E-posta'!$A$14:$D$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hesaplamalar'!$A$3:$C$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bildirim &amp; E-posta'!$A$14:$D$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Çıktılar &amp; Entegrasyon'!$A$3:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -604,7 +604,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1 — denetim içeriği + MUID + karşılık beyanı + GenAI/Agentic kategoriler</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +926,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Model riski panosu: KPI şeridi, tier dağılımı (donut), kategori dağılımı, validasyon takvimi, son kararlar</t>
+          <t>Model riski panosu: KPI şeridi (Süreçteki Validasyonlar + Periyodik Validasyonda dahil), tıklanabilir süreç paneli, tier dağılımı (donut), kategori dağılımı (Generative AI &amp; Agentic AI dahil), validasyon takvimi, son kararlar</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Banka geneli tüm modeller: birim×sınıf matrisi, filtreler (sınıf/tier/durum/birim/KAYNAK), gruplama, arama; İş Birimi Yeni Giriş (beyan), Yeni Model, CSV içe/dışa aktarma</t>
+          <t>Banka geneli tüm modeller: birim×sınıf matrisi, filtreler (sınıf/tier/durum/birim/KAYNAK), gruplama, arama (MUID dahil); İş Birimi Yeni Giriş (beyan), Yeni Model, CSV içe/dışa aktarma</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -1534,17 +1534,17 @@
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>Tüm işlemlerin zaman-rol-nesne kaydı (son 200); temizleme yalnız 2. Hat MRM</t>
+          <t>Tüm işlemlerin zaman-rol-nesne kaydı (son 200) + İçerik sütunu; satıra tıklanınca İŞLEM İÇERİĞİ draweri: alan-bazlı Önceki → Yeni değer tablosu (örn. Validasyon Frekansı: Yıllık → 2 Yıllık); temizleme yalnız 2. Hat MRM</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>Log tablosu</t>
+          <t>Log tablosu (tıklanır), içerik draweri</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
-          <t>History Log / Access History</t>
+          <t>History Log — field history (alan-seviyesi değişiklik geçmişi)</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2882,8 +2882,134 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>UC-27</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Karşılık Etkisi Beyanı</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>Beyan Anketi</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>1. Hat, 2. Hat MRM</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>Beyan formu açık</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>'⚠ Model karşılık etkisi yaratıyor' → popup: 'Tüm olası paydaşlar bilgilendirilecektir, kabul ediyor musunuz?' → Onayla / Geri Dön</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>Onayda işaret kaydedilir; Finansal Raporlama/IFRS9/MRM/Validasyon'a PROVISION-IMPACT bildirimi üretilir; Envanter Beyanı sekmesinde görünür</t>
+        </is>
+      </c>
+      <c r="H30" s="15" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>UC-28</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Denetim Kaydı İçeriği Görüntüle</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Denetim İzi</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Tüm roller (salt-okur dahil)</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Kayıtta içerik (chg) mevcut</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Denetim izinde satıra tıkla</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Drawer: işlem künyesi + Alan | Önceki → Yeni değişiklik tablosu (örn. valFrekans Yıllık → 2 Yıllık); LOG-##### kayıt no</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>UC-29</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>MUID ile Model Çağırma</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>Model Envanteri</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>Tüm roller</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>Arama kutusuna MUID yaz (HB-MDL-…) ya da sistemsel findModel(muid)</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>Model benzersiz-değiştirilemez kimliğiyle bulunur/açılır; MUID düzenlemeyle değişmez</t>
+        </is>
+      </c>
+      <c r="H32" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H29"/>
+  <autoFilter ref="A3:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2895,7 +3021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3408,23 +3534,23 @@
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>4 · Materyalite (S.03.A) — Gelişmiş</t>
+          <t>3 · Nitelikler &amp; Kritiklik</t>
         </is>
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>M1 — Risk tutarı / portföy büyüklüğü</t>
+          <t>Model karşılık etkisi yaratıyor (buton)</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>buton+popup</t>
         </is>
       </c>
       <c r="E19" s="16" t="inlineStr"/>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>Çok Düşük(1)…Çok Yüksek(5)</t>
+          <t>Popup: 'Tüm olası paydaşlar bilgilendirilecektir, kabul ediyor musunuz?' — Onayla/Geri Dön; onayda PROVISION-IMPACT bildirimi</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3567,7 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>M2 — Etkilenen müşteri/işlem sayısı</t>
+          <t>M1 — Risk tutarı / portföy büyüklüğü</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -3469,7 +3595,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>M3 — Kararlara etki</t>
+          <t>M2 — Etkilenen müşteri/işlem sayısı</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
@@ -3497,7 +3623,7 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>M4 — Ödeme gücü / yasal sermaye</t>
+          <t>M3 — Kararlara etki</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
@@ -3525,7 +3651,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>M5 — İtibar / davranışsal etki</t>
+          <t>M4 — Ödeme gücü / yasal sermaye</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -3548,12 +3674,12 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>5 · Karmaşıklık (S.03.B) — Gelişmiş</t>
+          <t>4 · Materyalite (S.03.A) — Gelişmiş</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>K1 — Girdi veri niteliği</t>
+          <t>M5 — İtibar / davranışsal etki</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
@@ -3581,7 +3707,7 @@
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>K2 — Metodoloji karmaşıklığı</t>
+          <t>K1 — Girdi veri niteliği</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -3609,7 +3735,7 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>K3 — Uygulama/entegrasyon</t>
+          <t>K2 — Metodoloji karmaşıklığı</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
@@ -3637,7 +3763,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>K4 — Kullanım sıklığı</t>
+          <t>K3 — Uygulama/entegrasyon</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -3665,7 +3791,7 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>K5 — Açıklanabilirlik/opaklık</t>
+          <t>K4 — Kullanım sıklığı</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
@@ -3693,7 +3819,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>K6 — Yanlılık potansiyeli</t>
+          <t>K5 — Açıklanabilirlik/opaklık</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -3721,7 +3847,7 @@
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>K7 — Otonomi/rekalibrasyon</t>
+          <t>K6 — Yanlılık potansiyeli</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
@@ -3744,12 +3870,12 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>5 · Karmaşıklık — Gelişmiş</t>
+          <t>5 · Karmaşıklık (S.03.B) — Gelişmiş</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>O1 — Otonomi düzeyi</t>
+          <t>K7 — Otonomi/rekalibrasyon</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -3760,7 +3886,7 @@
       <c r="E31" s="16" t="inlineStr"/>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>0-3 (Doğrudan karar seçilirse min 3)</t>
+          <t>Çok Düşük(1)…Çok Yüksek(5)</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3903,7 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>B1 — Downstream bağımlılık</t>
+          <t>O1 — Otonomi düzeyi</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
@@ -3788,7 +3914,7 @@
       <c r="E32" s="15" t="inlineStr"/>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-3 (Doğrudan karar seçilirse min 3)</t>
         </is>
       </c>
     </row>
@@ -3800,12 +3926,12 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>6 · Validasyon Takvimi</t>
+          <t>5 · Karmaşıklık — Gelişmiş</t>
         </is>
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Son validasyon ne zaman?</t>
+          <t>B1 — Downstream bağımlılık</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -3816,7 +3942,7 @@
       <c r="E33" s="16" t="inlineStr"/>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>Bu yıl · Geçen yıl · 2 yıl önce · Henüz yok</t>
+          <t>0-3</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3959,7 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Validasyon Frekansı</t>
+          <t>Son validasyon ne zaman?</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
@@ -3844,7 +3970,7 @@
       <c r="E34" s="15" t="inlineStr"/>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>Tier'dan otomatik · Yıllık · 2/3 Yıllık · Olay-Tetikli</t>
+          <t>Bu yıl · Geçen yıl · 2 yıl önce · Henüz yok</t>
         </is>
       </c>
     </row>
@@ -3856,21 +3982,25 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>7 · Resmi Halkbank Envanter Alanları — Gelişmiş</t>
+          <t>6 · Validasyon Takvimi</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Model Amacı (*)</t>
+          <t>Validasyon Frekansı</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>metin-uzun</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E35" s="16" t="inlineStr"/>
-      <c r="F35" s="16" t="inlineStr"/>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>Tier'dan otomatik · Yıllık · 2/3 Yıllık · Olay-Tetikli</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
@@ -3885,20 +4015,16 @@
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Kullanıldığı İş Süreci (NOTA Süreci vb.)</t>
+          <t>Model Amacı (*)</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>metin-uzun</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr"/>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>10 süreç</t>
-        </is>
-      </c>
+      <c r="F36" s="15" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -3913,7 +4039,7 @@
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Modelin İş Kararı Üzerindeki Etkisi</t>
+          <t>Kullanıldığı İş Süreci (NOTA Süreci vb.)</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -3924,7 +4050,7 @@
       <c r="E37" s="16" t="inlineStr"/>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Doğrudan karar · Karar destek · Bilgilendirme (Doğrudan→O1=3)</t>
+          <t>10 süreç</t>
         </is>
       </c>
     </row>
@@ -3941,7 +4067,7 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Model Türü</t>
+          <t>Modelin İş Kararı Üzerindeki Etkisi</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
@@ -3952,7 +4078,7 @@
       <c r="E38" s="15" t="inlineStr"/>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>İstatistiksel · Ekonometrik · ML · GenAI · Kural · Hibrit</t>
+          <t>Doğrudan karar · Karar destek · Bilgilendirme (Doğrudan→O1=3)</t>
         </is>
       </c>
     </row>
@@ -3969,7 +4095,7 @@
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Modelleme Yaklaşımı</t>
+          <t>Model Türü</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -3980,7 +4106,7 @@
       <c r="E39" s="16" t="inlineStr"/>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Denetimli/Denetimsiz/Zaman Serisi/Optimizasyon/Kural/Simülasyon</t>
+          <t>İstatistiksel · Ekonometrik · ML · GenAI · Kural · Hibrit</t>
         </is>
       </c>
     </row>
@@ -3997,7 +4123,7 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Geliştirildiği Platform</t>
+          <t>Modelleme Yaklaşımı</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -4008,7 +4134,7 @@
       <c r="E40" s="15" t="inlineStr"/>
       <c r="F40" s="15" t="inlineStr">
         <is>
-          <t>Dataiku · SPSS · SAS · Excel · MATLAB · Python · R · KNIME</t>
+          <t>Denetimli/Denetimsiz/Zaman Serisi/Optimizasyon/Kural/Simülasyon</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4151,7 @@
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>Model Geliştirmek için Kullanılan Dil</t>
+          <t>Geliştirildiği Platform</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -4036,7 +4162,7 @@
       <c r="E41" s="16" t="inlineStr"/>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Python · SQL · R · SAS · MATLAB · VBA · Scala</t>
+          <t>Dataiku · SPSS · SAS · Excel · MATLAB · Python · R · KNIME</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4179,7 @@
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Modede Kullanılan Algoritma</t>
+          <t>Model Geliştirmek için Kullanılan Dil</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -4064,7 +4190,7 @@
       <c r="E42" s="15" t="inlineStr"/>
       <c r="F42" s="15" t="inlineStr">
         <is>
-          <t>Loj.Reg · Karar Ağacı · RF · GBM · K-Means · NN · LLM …</t>
+          <t>Python · SQL · R · SAS · MATLAB · VBA · Scala</t>
         </is>
       </c>
     </row>
@@ -4081,16 +4207,20 @@
       </c>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>Modelleme Verisi Tarih Aralığı</t>
+          <t>Modede Kullanılan Algoritma</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>metin</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr"/>
-      <c r="F43" s="16" t="inlineStr"/>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>Loj.Reg · Karar Ağacı · RF · GBM · K-Means · NN · LLM …</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
@@ -4105,12 +4235,12 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Model Geliştirme Tarihi (**)</t>
+          <t>Modelleme Verisi Tarih Aralığı</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>tarih</t>
+          <t>metin</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr"/>
@@ -4129,7 +4259,7 @@
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Model Son Revizyon Tarihi (Yenileme/Kalibrasyon)</t>
+          <t>Model Geliştirme Tarihi (**)</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -4153,12 +4283,12 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Model Geliştiricisi (Birim/Bölüm veya Firma)</t>
+          <t>Model Son Revizyon Tarihi (Yenileme/Kalibrasyon)</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>metin</t>
+          <t>tarih</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr"/>
@@ -4177,7 +4307,7 @@
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Model Danışman Adı (danışmanlık alındıysa)</t>
+          <t>Model Geliştiricisi (Birim/Bölüm veya Firma)</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -4201,7 +4331,7 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Model Kullanıcısı Birim ve Bölümler</t>
+          <t>Model Danışman Adı (danışmanlık alındıysa)</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
@@ -4225,7 +4355,7 @@
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Model Hakkında İletişim Kurulacak Banka Personeli</t>
+          <t>Model Kullanıcısı Birim ve Bölümler</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -4234,11 +4364,7 @@
         </is>
       </c>
       <c r="E49" s="16" t="inlineStr"/>
-      <c r="F49" s="16" t="inlineStr">
-        <is>
-          <t>Model sahibi olarak da kullanılır</t>
-        </is>
-      </c>
+      <c r="F49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
@@ -4253,18 +4379,18 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Kontrol/Doğrulama süreci işletiliyor mu?</t>
+          <t>Model Hakkında İletişim Kurulacak Banka Personeli</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>metin</t>
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr"/>
       <c r="F50" s="15" t="inlineStr">
         <is>
-          <t>Evet/Hayır</t>
+          <t>Model sahibi olarak da kullanılır</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4407,7 @@
       </c>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>Performans ölçümü yapılıyor mu?</t>
+          <t>Kontrol/Doğrulama süreci işletiliyor mu?</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -4309,7 +4435,7 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>BDDK denetimi kapsamında mı?</t>
+          <t>Performans ölçümü yapılıyor mu?</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
@@ -4320,7 +4446,7 @@
       <c r="E52" s="15" t="inlineStr"/>
       <c r="F52" s="15" t="inlineStr">
         <is>
-          <t>Evet → düzenleyici işaretlenir (Tier'ı etkiler)</t>
+          <t>Evet/Hayır</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4463,7 @@
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>İç denetim kapsamında mı?</t>
+          <t>BDDK denetimi kapsamında mı?</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -4348,7 +4474,7 @@
       <c r="E53" s="16" t="inlineStr"/>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>Evet/Hayır</t>
+          <t>Evet → düzenleyici işaretlenir (Tier'ı etkiler)</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4491,7 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Model dokümanı bulunuyor mu?</t>
+          <t>İç denetim kapsamında mı?</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
@@ -4393,36 +4519,40 @@
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Açıklama (Opsiyonel) (***)</t>
+          <t>Model dokümanı bulunuyor mu?</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>metin-uzun</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr"/>
-      <c r="F55" s="16" t="inlineStr"/>
+      <c r="F55" s="16" t="inlineStr">
+        <is>
+          <t>Evet/Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="15" t="inlineStr">
         <is>
-          <t>Model Formu (uzman)</t>
+          <t>Beyan Anketi</t>
         </is>
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>(özet)</t>
+          <t>7 · Resmi Halkbank Envanter Alanları — Gelişmiş</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Ad*, Tip, Sınıf, Amaç, Kategori(çoklu), Bayraklar(AI/GenAI/Det/Düzenleyici), Köken, Tedarikçi, Birim, Sahip, Geliştirici, Validatör, Metodoloji, Algoritma, Sistem, Durum, 3 tarih, Frekans, Varsayım/Sınırlama, 4 link, Upstream(çoklu)</t>
+          <t>Açıklama (Opsiyonel) (***)</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
         <is>
-          <t>karma</t>
+          <t>metin-uzun</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr"/>
@@ -4431,7 +4561,7 @@
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>Validasyon Formu</t>
+          <t>Model Formu (uzman)</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
@@ -4441,7 +4571,7 @@
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>Başlık*, Model*, Tür(6), Tetik(6), Validatör, Bağımsızlık(4), Backtest, Ayrım Gücü, Etkin Sorgulama, ÖNERİ(3), Rating(3), Rapor Tarihi, ONAY kararı(4)+Makam — onay alanları yalnız Komite rolünde aktif</t>
+          <t>Ad*, Tip, Sınıf, Amaç, Kategori(çoklu), Bayraklar(AI/GenAI/Det/Düzenleyici), Köken, Tedarikçi, Birim, Sahip, Geliştirici, Validatör, Metodoloji, Algoritma, Sistem, Durum, 3 tarih, Frekans, Varsayım/Sınırlama, 4 link, Upstream(çoklu)</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -4455,7 +4585,7 @@
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
-          <t>Bulgu / Remediation Formu</t>
+          <t>Validasyon Formu</t>
         </is>
       </c>
       <c r="B58" s="15" t="inlineStr">
@@ -4465,7 +4595,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Başlık*, Model, Kaynak(5), Önem(3→SLA), Remediation Durumu(6 aşama), Sorumlu, 2 tarih, Aksiyon Planı, Kanıt/Re-test — kapanış onay bloğu yalnız 2. hat</t>
+          <t>Başlık*, Model*, Tür(6), Tetik(6), Validatör, Bağımsızlık(4), Backtest, Ayrım Gücü, Etkin Sorgulama, ÖNERİ(3), Rating(3), Rapor Tarihi, ONAY kararı(4)+Makam — onay alanları yalnız Komite rolünde aktif</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
@@ -4479,7 +4609,7 @@
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>Overlay / İstisna Formu</t>
+          <t>Bulgu / Remediation Formu</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
@@ -4489,7 +4619,7 @@
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>Model*, Tür(5), Materyalite, Etki Yönü, Etki Tutarı, TFRS9 Aşaması, Senaryo, Gerekçe, Hesaplama, Kaldırma Kriteri, Onay Makamı, Bağımsız G.G.(4), Durum + Komite onay düğmeleri</t>
+          <t>Başlık*, Model, Kaynak(5), Önem(3→SLA), Remediation Durumu(6 aşama), Sorumlu, 2 tarih, Aksiyon Planı, Kanıt/Re-test — kapanış onay bloğu yalnız 2. hat</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -4503,7 +4633,7 @@
     <row r="60">
       <c r="A60" s="15" t="inlineStr">
         <is>
-          <t>Guardrail Test Formu</t>
+          <t>Overlay / İstisna Formu</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
@@ -4513,7 +4643,7 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Model(GenAI)*, Test Türü(7), Tarih, Sonuç(Geçti/Kaldı), Şiddet, Detay — 'Kaldı' otomatik bulgu</t>
+          <t>Model*, Tür(5), Materyalite, Etki Yönü, Etki Tutarı, TFRS9 Aşaması, Senaryo, Gerekçe, Hesaplama, Kaldırma Kriteri, Onay Makamı, Bağımsız G.G.(4), Durum + Komite onay düğmeleri</t>
         </is>
       </c>
       <c r="D60" s="15" t="inlineStr">
@@ -4527,7 +4657,7 @@
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>Vendor Formu</t>
+          <t>Guardrail Test Formu</t>
         </is>
       </c>
       <c r="B61" s="16" t="inlineStr">
@@ -4537,7 +4667,7 @@
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Tedarikçi, Şeffaflık(kara/gri/şeffaf), SLA, Çıkış Stratejisi, Kara-kutu Kısıtı, Due-Diligence(3), Son Gözden Geçirme</t>
+          <t>Model(GenAI)*, Test Türü(7), Tarih, Sonuç(Geçti/Kaldı), Şiddet, Detay — 'Kaldı' otomatik bulgu</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -4551,7 +4681,7 @@
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t>Faz Formu (Model Journey)</t>
+          <t>Vendor Formu</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
@@ -4561,7 +4691,7 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Faz başına R_Sxx_n alanları (dropdown/metin/sayı/tarih; * zorunlu) — 10 faz × 3-5 alan; kayıt ilerlemeyi besler</t>
+          <t>Tedarikçi, Şeffaflık(kara/gri/şeffaf), SLA, Çıkış Stratejisi, Kara-kutu Kısıtı, Due-Diligence(3), Son Gözden Geçirme</t>
         </is>
       </c>
       <c r="D62" s="15" t="inlineStr">
@@ -4572,8 +4702,32 @@
       <c r="E62" s="15" t="inlineStr"/>
       <c r="F62" s="15" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>Faz Formu (Model Journey)</t>
+        </is>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>(özet)</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Faz başına R_Sxx_n alanları (dropdown/metin/sayı/tarih; * zorunlu) — 10 faz × 3-5 alan; kayıt ilerlemeyi besler</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>karma</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr"/>
+      <c r="F63" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F62"/>
+  <autoFilter ref="A3:F63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4643,7 +4797,7 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>id (MDL-####), ad, tip, sinif, modelTipi, kategori[], amac, amacDetay, metricProfile, aiml, genai, deterministik, duzenleyici, koken, tedarikci, sahipBirim, sahip, gelistirici, validator, metodoloji, algoritma, barindiran, durum, durumTalep, wf (mrm/komite/aktif/red), gelistirmeTarihi, prodTarihi, sonValidasyon, valFrekans, izlemeDurumu, upstream[], links{doc,monitor,repo,val}, kaynak, crit{M1-M5,K1-K7,B1,O1,duzenleyici,genai}, mat, kar, icsel, tier, derece, envanter{23 resmi alan,_auto}, vendor{}, phases[10], aimlEk{}, lifecyclePhase</t>
+          <t>id (MDL-####), muid (HB-MDL-XXXXXXXXXXXX — benzersiz, DEĞİŞTİRİLEMEZ; oluşturmada atanır, düzenlemede korunur), karsilikEtkisi, ad, tip, sinif, modelTipi, kategori[], amac, amacDetay, metricProfile, aiml, genai, deterministik, duzenleyici, koken, tedarikci, sahipBirim, sahip, gelistirici, validator, metodoloji, algoritma, barindiran, durum, durumTalep, wf (mrm/komite/aktif/red), gelistirmeTarihi, prodTarihi, sonValidasyon, valFrekans, izlemeDurumu, upstream[], links{doc,monitor,repo,val}, kaynak, crit{M1-M5,K1-K7,B1,O1,duzenleyici,genai}, mat, kar, icsel, tier, derece, envanter{23 resmi alan,_auto}, vendor{}, phases[10], aimlEk{}, lifecyclePhase</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
@@ -4797,12 +4951,12 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>ts, role, action, entity, detail (max 500)</t>
+          <t>aid (LOG-#####), ts, role, action, entity, detail, chg[] = alan-bazlı değişiklik içeriği {alan, eski, yeni} (max 500 kayıt)</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>History Log</t>
+          <t>History Log + field history</t>
         </is>
       </c>
     </row>
@@ -5509,7 +5663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5857,22 +6011,39 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
+          <t>MUID üretimi</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>HB-MDL- + 12 hex (crypto.getRandomValues); oluşturmada atanır; saveModel düzenlemede önceki değeri zorla korur</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Değiştirilemezlik uygulama katmanında garanti edilir; Archer'da key field (read-only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
           <t>Metrik üretimi</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Model çerçevesine göre son 6 ay (dinamik) seri; _degrade işaretli modellerde son 2 ay eşik ihlali</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>Beyan/CSV modellerinde otomatik</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C22"/>
+  <autoFilter ref="A3:C23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5884,7 +6055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6232,36 +6403,58 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
+          <t>Karşılık etkisi beyanı</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Finansal Raporlama + IFRS9 Ekibi + MRM + Validasyon</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>PROVISION-IMPACT</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Anında</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
           <t>Haftalık MRM yönetim özeti</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>MRM Programı + Üst Yönetim</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>WEEKLY-DIGEST</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Haftalık (Pzt 08:00)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Talep: Bu kurallar Archer Notifications + Advanced Workflow notification şablonları ve scheduled report/digest ile e-posta olarak uygulanacaktır. Uygulamada giden kutusu simülasyonu ve günlük özet önizlemesi (mailto) mevcuttur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A14:D21"/>
+  <autoFilter ref="A14:D22"/>
   <mergeCells count="1">
-    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6354,7 +6547,7 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Model Adı, İş Birimi, Sınıf, Model Tipi, Kategori, Durum, Metrik Çerçevesi, Düzenleyici, AI/ML, Genel Kritiklik, Son Validasyon, Tier, İçsel Risk, Kaynak</t>
+          <t>Model ID, MUID, Model Adı, İş Birimi, Sınıf, Model Tipi, Kategori, Durum, Metrik Çerçevesi, Düzenleyici, AI/ML, Genel Kritiklik, Son Validasyon, Tier, İçsel Risk, Kaynak</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Dokuman: tanitim Excel v1.2 — bolumlu Yeni Model formu, iliski panelleri (UC-30), NOTA (UC-31), zorunlu gerekce (UC-32), dikey liste duzeni, surum URL'leri
</commit_message>
<xml_diff>
--- a/mrm-archer/MRM_Konsolu_Yazilim_Tanitim.xlsx
+++ b/mrm-archer/MRM_Konsolu_Yazilim_Tanitim.xlsx
@@ -19,8 +19,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Menü Envanteri'!$A$3:$F$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'İşlemler (Use-Case)'!$A$3:$H$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Formlar &amp; Alanlar'!$A$3:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'İşlemler (Use-Case)'!$A$3:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Formlar &amp; Alanlar'!$A$3:$F$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Veri Modeli'!$A$3:$D$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roller &amp; Yetki'!$A$3:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hesaplamalar'!$A$3:$C$23</definedName>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -604,7 +604,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>v1.1 — denetim içeriği + MUID + karşılık beyanı + GenAI/Agentic kategoriler</t>
+          <t>v1.2 — bölümlü Yeni Model formu + upstream/downstream ilişki panelleri + NOTA süreci + zorunlu ihtiyaç gerekçesi</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -659,179 +659,191 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Hedef Platform</t>
+          <t>Sürüm Geri Dönüş (rollback)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>RSA Archer (IRM) — her özellik ilgili Archer mekanizmasıyla eşlenmiştir</t>
+          <t>v1: /mrm/v1/ · v2: /mrm/v2/ (kalıcı URL kopyaları) + yerel git tag'leri mrm-v1.0 / mrm-v2.0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>Hedef Platform</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>RSA Archer (IRM) — her özellik ilgili Archer mekanizmasıyla eşlenmiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>Kapsam Notu</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Uygulama tarayıcıda (localStorage) çalışan bir simülasyondur; bu doküman Archer'da geliştirilecek yapının işlevsel tarifidir.</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>SAYFA KILAVUZU</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Sayfa</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>İçerik</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Menü Envanteri</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>24 menü/ekranın amacı, bileşenleri ve Archer karşılığı</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>İşlemler (Use-Case)</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Tüm kullanıcı işlemleri: aktör, ön koşul, akış, sonuç, denetim izi</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Formlar &amp; Alanlar</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Beyan anketi (7 bölüm) ve tüm form alanları: tip, zorunluluk, seçenekler</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Veri Modeli</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>state varlıkları ve alan sözlüğü</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Roller &amp; Yetki</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Rol × işlem matrisi + özel yetki kuralları (görevler ayrılığı)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Hesaplamalar</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Kritiklik/Tier skoru, TMR endeksi, SLA, frekans, metrik eşikleri, İSEDES eşleme</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Bildirim &amp; E-posta</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Kural motoru + Archer Notifications e-posta talebi (7 kural)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Çıktılar &amp; Entegrasyon</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>XLSX (10 sheet), CSV içe/dışa, JSON, BDDK paketi, mailto</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Özet sayılar (üretim betiğince sayılmıştır — statik doküman):</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Menü sayısı</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="n">
-        <v>25</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Tanımlı işlem sayısı</t>
+          <t>Menü sayısı</t>
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>Tanımlı işlem sayısı</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>Form alanı sayısı</t>
         </is>
       </c>
-      <c r="B28" s="12" t="n">
-        <v>60</v>
+      <c r="B29" s="12" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1054,12 +1066,12 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Banka geneli tüm modeller: birim×sınıf matrisi, filtreler (sınıf/tier/durum/birim/KAYNAK), gruplama, arama (MUID dahil); İş Birimi Yeni Giriş (beyan), Yeni Model, CSV içe/dışa aktarma</t>
+          <t>Banka geneli tüm modeller: birim×sınıf matrisi, filtreler (sınıf/tier/durum/birim/KAYNAK), gruplama, arama (MUID dahil); İş Birimi Yeni Giriş (beyan; ZORUNLU Model İhtiyacı Gerekçesi), Yeni Model (7 bölümlü uzman formu: kategori/bayraklar dikey liste + Seçilenler kutusu, NOTA süreci, upstream/downstream ilişki panelleri), CSV içe/dışa aktarma</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>Matris tablo, filtre çubuğu, model tablosu, model detay drawer (8 sekme)</t>
+          <t>Matris tablo, filtre çubuğu, model tablosu, model detay drawer (8 sekme), ilişki panelleri (rel-list + rel-side)</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -1438,7 +1450,7 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Model bağımlılık ağı (upstream/downstream), özyinelemeli etki analizi ('bu model bozulursa')</t>
+          <t>Model bağımlılık ağı (upstream/downstream — Yeni Model formundaki ilişki panellerinden beslenir, çift yönlü), özyinelemeli etki analizi; seçili modelin İlişkili NOTA Süreci callout'u</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
@@ -1721,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1840,7 +1852,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Yeni Model (uzman formu)</t>
+          <t>Yeni Model (bölümlü uzman formu)</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -1860,12 +1872,12 @@
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>'+ Yeni Model' → tam form → Kaydet</t>
+          <t>'+ Yeni Model' → 7 bölümlü form (Kimlik / Tanım / Bayraklar-liste / NOTA / İlişkilendirme / Tarihler / Dokümantasyon); Kategori ve Bayraklar dikey liste + yanda 'Seçilenler' kutusu</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>UC-01 ile aynı onay akışına girer (wf=MRM, durum=Onayda, İlk Validasyon kaydı)</t>
+          <t>UC-01 ile aynı onay akışına girer (wf=MRM, durum=Onayda, İlk Validasyon kaydı); metrik çerçevesi seçildiyse izleme serisi üretilir</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
@@ -3008,8 +3020,134 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>UC-30</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Bağımlılık İlişkilendirme (Upstream/Downstream)</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Yeni Model / Model Düzenle</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>1. Hat, 2. Hat MRM</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>Bölüm 5: iki ayrı panel (⬆ Besleyen / ⬇ Beslenen) — listeden tik at, seçilenler yandaki kutuda canlı görünür → Kaydet</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Downstream seçimi karşı modelin upstream kaydına ÇİFT YÖNLÜ işlenir; Bağımlılık &amp; Etki ağ grafiğine anında yansır; 'Bağımlılık ilişkilendirme' denetim kaydı İÇERİKLİ (önceki → yeni ilişki listeleri) düşer</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>UC-31</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>NOTA Süreç İlişkilendirme</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Yeni Model / Model Düzenle</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>1. Hat, 2. Hat MRM</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>Bölüm 4: 'İlişkili NOTA Süreci' dropdown (22 kayıtlık banka süreç kataloğu, akademik tez numaralandırması: 1.1.1. Bireysel Kredi Tahsis…)</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>Model NOTA sürecine bağlanır; model detayı Genel sekmesinde ve Bağımlılık &amp; Etki sayfasında 📌 callout olarak görünür (Archer NOTA ekranı cross-reference)</t>
+        </is>
+      </c>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>UC-32</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Model İhtiyacı Gerekçesi (zorunlu)</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Beyan Anketi</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>1. Hat, 2. Hat MRM</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>Bölüm 1: 'Model İhtiyacı Gerekçesi — bu modele neden ihtiyaç duyuldu?' zorunlu açıklama</t>
+        </is>
+      </c>
+      <c r="G35" s="16" t="inlineStr">
+        <is>
+          <t>Boş bırakılırsa kayıt engellenir; model + resmi envanter kaydına işlenir, detay ve Envanter Beyanı sekmesinde gösterilir</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H32"/>
+  <autoFilter ref="A3:H35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3021,7 +3159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3119,12 +3257,12 @@
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Beyan Eden İş Birimi</t>
+          <t>Model İhtiyacı Gerekçesi (neden doğdu?)</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>metin-uzun</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
@@ -3134,7 +3272,7 @@
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>10 GMY/Başkanlık</t>
+          <t>ZORUNLU — boşsa kayıt engellenir</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3289,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Köken</t>
+          <t>Beyan Eden İş Birimi</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -3159,10 +3297,14 @@
           <t>dropdown</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr"/>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>İç Geliştirme · Satıcı/Vendor · Grup-Ana Model</t>
+          <t>10 GMY/Başkanlık</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3321,7 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Model Durumu</t>
+          <t>Köken</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
@@ -3187,14 +3329,10 @@
           <t>dropdown</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
+      <c r="E7" s="16" t="inlineStr"/>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>Geliştirme · Validasyonda · Onaylı/Prod · İzlemede</t>
+          <t>İç Geliştirme · Satıcı/Vendor · Grup-Ana Model</t>
         </is>
       </c>
     </row>
@@ -3206,12 +3344,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>2 · Model Tanımı (PMJ)</t>
+          <t>1 · Kimlik &amp; Sahiplik</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Model Sınıfı</t>
+          <t>Model Durumu</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -3226,7 +3364,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Geleneksel · Ekonometrik · ML/AI</t>
+          <t>Geliştirme · Validasyonda · Onaylı/Prod · İzlemede</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3381,7 @@
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Model Tipi</t>
+          <t>Model Sınıfı</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -3258,7 +3396,7 @@
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>İLERİ ANALİTİK MODEL · BASİT MODEL</t>
+          <t>Geleneksel · Ekonometrik · ML/AI</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3413,7 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Model Kategorisi</t>
+          <t>Model Tipi</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -3290,7 +3428,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Kredi/IRB, TFRS9, VaR, IRRBB, AML… (10)</t>
+          <t>İLERİ ANALİTİK MODEL · BASİT MODEL</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3445,7 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Amaç / Kullanım</t>
+          <t>Model Kategorisi</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
@@ -3322,7 +3460,7 @@
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>12 amaç</t>
+          <t>Kredi/IRB, TFRS9, VaR, IRRBB, AML… (10)</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3477,7 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Metodoloji Ailesi</t>
+          <t>Amaç / Kullanım</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -3347,10 +3485,14 @@
           <t>dropdown</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>11 metodoloji</t>
+          <t>12 amaç</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3509,7 @@
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>Performans Metrik Çerçevesi</t>
+          <t>Metodoloji Ailesi</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
@@ -3375,14 +3517,10 @@
           <t>dropdown</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
+      <c r="E13" s="16" t="inlineStr"/>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>10 çerçeve — izleme metriklerini belirler</t>
+          <t>11 metodoloji</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3537,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Yaşam Döngüsü Fazı</t>
+          <t>Performans Metrik Çerçevesi</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
@@ -3407,10 +3545,14 @@
           <t>dropdown</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>4 faz (LC4)</t>
+          <t>10 çerçeve — izleme metriklerini belirler</t>
         </is>
       </c>
     </row>
@@ -3422,12 +3564,12 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>3 · Nitelikler &amp; Kritiklik</t>
+          <t>2 · Model Tanımı (PMJ)</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>AI/ML modeli mi?</t>
+          <t>Yaşam Döngüsü Fazı</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -3438,7 +3580,7 @@
       <c r="E15" s="16" t="inlineStr"/>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>Evet/Hayır</t>
+          <t>4 faz (LC4)</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3597,7 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>GenAI / Temel Model mi?</t>
+          <t>AI/ML modeli mi?</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
@@ -3483,7 +3625,7 @@
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>Düzenleyici / sermaye kullanımı?</t>
+          <t>GenAI / Temel Model mi?</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
@@ -3511,7 +3653,7 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Genel Kritiklik Düzeyi</t>
+          <t>Düzenleyici / sermaye kullanımı?</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
@@ -3522,7 +3664,7 @@
       <c r="E18" s="15" t="inlineStr"/>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>Düşük · Orta · Yüksek · Kritik (basit mod; boşsa 'Orta' varsayılır)</t>
+          <t>Evet/Hayır</t>
         </is>
       </c>
     </row>
@@ -3539,18 +3681,18 @@
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>Model karşılık etkisi yaratıyor (buton)</t>
+          <t>Genel Kritiklik Düzeyi</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>buton+popup</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E19" s="16" t="inlineStr"/>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>Popup: 'Tüm olası paydaşlar bilgilendirilecektir, kabul ediyor musunuz?' — Onayla/Geri Dön; onayda PROVISION-IMPACT bildirimi</t>
+          <t>Düşük · Orta · Yüksek · Kritik (basit mod; boşsa 'Orta' varsayılır)</t>
         </is>
       </c>
     </row>
@@ -3562,23 +3704,23 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>4 · Materyalite (S.03.A) — Gelişmiş</t>
+          <t>3 · Nitelikler &amp; Kritiklik</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>M1 — Risk tutarı / portföy büyüklüğü</t>
+          <t>Model karşılık etkisi yaratıyor (buton)</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>buton+popup</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr"/>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Çok Düşük(1)…Çok Yüksek(5)</t>
+          <t>Popup: 'Tüm olası paydaşlar bilgilendirilecektir, kabul ediyor musunuz?' — Onayla/Geri Dön; onayda PROVISION-IMPACT bildirimi</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3737,7 @@
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>M2 — Etkilenen müşteri/işlem sayısı</t>
+          <t>M1 — Risk tutarı / portföy büyüklüğü</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
@@ -3623,7 +3765,7 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>M3 — Kararlara etki</t>
+          <t>M2 — Etkilenen müşteri/işlem sayısı</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
@@ -3651,7 +3793,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>M4 — Ödeme gücü / yasal sermaye</t>
+          <t>M3 — Kararlara etki</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -3679,7 +3821,7 @@
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>M5 — İtibar / davranışsal etki</t>
+          <t>M4 — Ödeme gücü / yasal sermaye</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
@@ -3702,12 +3844,12 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>5 · Karmaşıklık (S.03.B) — Gelişmiş</t>
+          <t>4 · Materyalite (S.03.A) — Gelişmiş</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>K1 — Girdi veri niteliği</t>
+          <t>M5 — İtibar / davranışsal etki</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -3735,7 +3877,7 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>K2 — Metodoloji karmaşıklığı</t>
+          <t>K1 — Girdi veri niteliği</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
@@ -3763,7 +3905,7 @@
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>K3 — Uygulama/entegrasyon</t>
+          <t>K2 — Metodoloji karmaşıklığı</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -3791,7 +3933,7 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>K4 — Kullanım sıklığı</t>
+          <t>K3 — Uygulama/entegrasyon</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
@@ -3819,7 +3961,7 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>K5 — Açıklanabilirlik/opaklık</t>
+          <t>K4 — Kullanım sıklığı</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -3847,7 +3989,7 @@
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>K6 — Yanlılık potansiyeli</t>
+          <t>K5 — Açıklanabilirlik/opaklık</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
@@ -3875,7 +4017,7 @@
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>K7 — Otonomi/rekalibrasyon</t>
+          <t>K6 — Yanlılık potansiyeli</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -3898,12 +4040,12 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>5 · Karmaşıklık — Gelişmiş</t>
+          <t>5 · Karmaşıklık (S.03.B) — Gelişmiş</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>O1 — Otonomi düzeyi</t>
+          <t>K7 — Otonomi/rekalibrasyon</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
@@ -3914,7 +4056,7 @@
       <c r="E32" s="15" t="inlineStr"/>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>0-3 (Doğrudan karar seçilirse min 3)</t>
+          <t>Çok Düşük(1)…Çok Yüksek(5)</t>
         </is>
       </c>
     </row>
@@ -3931,7 +4073,7 @@
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>B1 — Downstream bağımlılık</t>
+          <t>O1 — Otonomi düzeyi</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -3942,7 +4084,7 @@
       <c r="E33" s="16" t="inlineStr"/>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-3 (Doğrudan karar seçilirse min 3)</t>
         </is>
       </c>
     </row>
@@ -3954,12 +4096,12 @@
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>6 · Validasyon Takvimi</t>
+          <t>5 · Karmaşıklık — Gelişmiş</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Son validasyon ne zaman?</t>
+          <t>B1 — Downstream bağımlılık</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
@@ -3970,7 +4112,7 @@
       <c r="E34" s="15" t="inlineStr"/>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>Bu yıl · Geçen yıl · 2 yıl önce · Henüz yok</t>
+          <t>0-3</t>
         </is>
       </c>
     </row>
@@ -3987,7 +4129,7 @@
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Validasyon Frekansı</t>
+          <t>Son validasyon ne zaman?</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -3998,7 +4140,7 @@
       <c r="E35" s="16" t="inlineStr"/>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>Tier'dan otomatik · Yıllık · 2/3 Yıllık · Olay-Tetikli</t>
+          <t>Bu yıl · Geçen yıl · 2 yıl önce · Henüz yok</t>
         </is>
       </c>
     </row>
@@ -4010,21 +4152,25 @@
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>7 · Resmi Halkbank Envanter Alanları — Gelişmiş</t>
+          <t>6 · Validasyon Takvimi</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Model Amacı (*)</t>
+          <t>Validasyon Frekansı</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
-          <t>metin-uzun</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr"/>
-      <c r="F36" s="15" t="inlineStr"/>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>Tier'dan otomatik · Yıllık · 2/3 Yıllık · Olay-Tetikli</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -4039,20 +4185,16 @@
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Kullanıldığı İş Süreci (NOTA Süreci vb.)</t>
+          <t>Model Amacı (*)</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>metin-uzun</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr"/>
-      <c r="F37" s="16" t="inlineStr">
-        <is>
-          <t>10 süreç</t>
-        </is>
-      </c>
+      <c r="F37" s="16" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
@@ -4067,7 +4209,7 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Modelin İş Kararı Üzerindeki Etkisi</t>
+          <t>Kullanıldığı İş Süreci (NOTA Süreci vb.)</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
@@ -4078,7 +4220,7 @@
       <c r="E38" s="15" t="inlineStr"/>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>Doğrudan karar · Karar destek · Bilgilendirme (Doğrudan→O1=3)</t>
+          <t>10 süreç</t>
         </is>
       </c>
     </row>
@@ -4095,7 +4237,7 @@
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Model Türü</t>
+          <t>Modelin İş Kararı Üzerindeki Etkisi</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -4106,7 +4248,7 @@
       <c r="E39" s="16" t="inlineStr"/>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>İstatistiksel · Ekonometrik · ML · GenAI · Kural · Hibrit</t>
+          <t>Doğrudan karar · Karar destek · Bilgilendirme (Doğrudan→O1=3)</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4265,7 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Modelleme Yaklaşımı</t>
+          <t>Model Türü</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
@@ -4134,7 +4276,7 @@
       <c r="E40" s="15" t="inlineStr"/>
       <c r="F40" s="15" t="inlineStr">
         <is>
-          <t>Denetimli/Denetimsiz/Zaman Serisi/Optimizasyon/Kural/Simülasyon</t>
+          <t>İstatistiksel · Ekonometrik · ML · GenAI · Kural · Hibrit</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4293,7 @@
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>Geliştirildiği Platform</t>
+          <t>Modelleme Yaklaşımı</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -4162,7 +4304,7 @@
       <c r="E41" s="16" t="inlineStr"/>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Dataiku · SPSS · SAS · Excel · MATLAB · Python · R · KNIME</t>
+          <t>Denetimli/Denetimsiz/Zaman Serisi/Optimizasyon/Kural/Simülasyon</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4321,7 @@
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Model Geliştirmek için Kullanılan Dil</t>
+          <t>Geliştirildiği Platform</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -4190,7 +4332,7 @@
       <c r="E42" s="15" t="inlineStr"/>
       <c r="F42" s="15" t="inlineStr">
         <is>
-          <t>Python · SQL · R · SAS · MATLAB · VBA · Scala</t>
+          <t>Dataiku · SPSS · SAS · Excel · MATLAB · Python · R · KNIME</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4349,7 @@
       </c>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>Modede Kullanılan Algoritma</t>
+          <t>Model Geliştirmek için Kullanılan Dil</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -4218,7 +4360,7 @@
       <c r="E43" s="16" t="inlineStr"/>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Loj.Reg · Karar Ağacı · RF · GBM · K-Means · NN · LLM …</t>
+          <t>Python · SQL · R · SAS · MATLAB · VBA · Scala</t>
         </is>
       </c>
     </row>
@@ -4235,16 +4377,20 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Modelleme Verisi Tarih Aralığı</t>
+          <t>Modede Kullanılan Algoritma</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>metin</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr"/>
-      <c r="F44" s="15" t="inlineStr"/>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Loj.Reg · Karar Ağacı · RF · GBM · K-Means · NN · LLM …</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -4259,12 +4405,12 @@
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Model Geliştirme Tarihi (**)</t>
+          <t>Modelleme Verisi Tarih Aralığı</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>tarih</t>
+          <t>metin</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr"/>
@@ -4283,7 +4429,7 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Model Son Revizyon Tarihi (Yenileme/Kalibrasyon)</t>
+          <t>Model Geliştirme Tarihi (**)</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
@@ -4307,12 +4453,12 @@
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Model Geliştiricisi (Birim/Bölüm veya Firma)</t>
+          <t>Model Son Revizyon Tarihi (Yenileme/Kalibrasyon)</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>metin</t>
+          <t>tarih</t>
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr"/>
@@ -4331,7 +4477,7 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Model Danışman Adı (danışmanlık alındıysa)</t>
+          <t>Model Geliştiricisi (Birim/Bölüm veya Firma)</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
@@ -4355,7 +4501,7 @@
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Model Kullanıcısı Birim ve Bölümler</t>
+          <t>Model Danışman Adı (danışmanlık alındıysa)</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -4379,7 +4525,7 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Model Hakkında İletişim Kurulacak Banka Personeli</t>
+          <t>Model Kullanıcısı Birim ve Bölümler</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
@@ -4388,11 +4534,7 @@
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr"/>
-      <c r="F50" s="15" t="inlineStr">
-        <is>
-          <t>Model sahibi olarak da kullanılır</t>
-        </is>
-      </c>
+      <c r="F50" s="15" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
@@ -4407,18 +4549,18 @@
       </c>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>Kontrol/Doğrulama süreci işletiliyor mu?</t>
+          <t>Model Hakkında İletişim Kurulacak Banka Personeli</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>metin</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr"/>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>Evet/Hayır</t>
+          <t>Model sahibi olarak da kullanılır</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4577,7 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Performans ölçümü yapılıyor mu?</t>
+          <t>Kontrol/Doğrulama süreci işletiliyor mu?</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
@@ -4463,7 +4605,7 @@
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>BDDK denetimi kapsamında mı?</t>
+          <t>Performans ölçümü yapılıyor mu?</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -4474,7 +4616,7 @@
       <c r="E53" s="16" t="inlineStr"/>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>Evet → düzenleyici işaretlenir (Tier'ı etkiler)</t>
+          <t>Evet/Hayır</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4633,7 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>İç denetim kapsamında mı?</t>
+          <t>BDDK denetimi kapsamında mı?</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
@@ -4502,7 +4644,7 @@
       <c r="E54" s="15" t="inlineStr"/>
       <c r="F54" s="15" t="inlineStr">
         <is>
-          <t>Evet/Hayır</t>
+          <t>Evet → düzenleyici işaretlenir (Tier'ı etkiler)</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4661,7 @@
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Model dokümanı bulunuyor mu?</t>
+          <t>İç denetim kapsamında mı?</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -4547,36 +4689,40 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Açıklama (Opsiyonel) (***)</t>
+          <t>Model dokümanı bulunuyor mu?</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
         <is>
-          <t>metin-uzun</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr"/>
-      <c r="F56" s="15" t="inlineStr"/>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>Evet/Hayır</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>Model Formu (uzman)</t>
+          <t>Beyan Anketi</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>(özet)</t>
+          <t>7 · Resmi Halkbank Envanter Alanları — Gelişmiş</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>Ad*, Tip, Sınıf, Amaç, Kategori(çoklu), Bayraklar(AI/GenAI/Det/Düzenleyici), Köken, Tedarikçi, Birim, Sahip, Geliştirici, Validatör, Metodoloji, Algoritma, Sistem, Durum, 3 tarih, Frekans, Varsayım/Sınırlama, 4 link, Upstream(çoklu)</t>
+          <t>Açıklama (Opsiyonel) (***)</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>karma</t>
+          <t>metin-uzun</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr"/>
@@ -4585,7 +4731,7 @@
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
-          <t>Validasyon Formu</t>
+          <t>Model Formu (uzman, 7 bölüm)</t>
         </is>
       </c>
       <c r="B58" s="15" t="inlineStr">
@@ -4595,7 +4741,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Başlık*, Model*, Tür(6), Tetik(6), Validatör, Bağımsızlık(4), Backtest, Ayrım Gücü, Etkin Sorgulama, ÖNERİ(3), Rating(3), Rapor Tarihi, ONAY kararı(4)+Makam — onay alanları yalnız Komite rolünde aktif</t>
+          <t>B1 Kimlik: Ad*, Sahip Birim(dropdown), Sahip, Köken, Tedarikçi, Durum, Geliştirici, Validatör · B2 Tanım: Tip, Sınıf, Metrik Çerçevesi(dropdown), Metodoloji, Algoritma, Sistem, Amaç, Kategori(DİKEY LİSTE + Seçilenler kutusu) · B3 Bayraklar(açıklamalı dikey liste) · B4 İlişkili NOTA Süreci(dropdown, 22 süreç) · B5 İlişkilendirme: Upstream &amp; Downstream AYRI paneller (tik + yanda Seçilenler kutusu; downstream ters-yazma) · B6 Tarihler &amp; Frekans · B7 Varsayım/Sınırlama + 4 link</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
@@ -4609,7 +4755,7 @@
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>Bulgu / Remediation Formu</t>
+          <t>Validasyon Formu</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
@@ -4619,7 +4765,7 @@
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>Başlık*, Model, Kaynak(5), Önem(3→SLA), Remediation Durumu(6 aşama), Sorumlu, 2 tarih, Aksiyon Planı, Kanıt/Re-test — kapanış onay bloğu yalnız 2. hat</t>
+          <t>Başlık*, Model*, Tür(6), Tetik(6), Validatör, Bağımsızlık(4), Backtest, Ayrım Gücü, Etkin Sorgulama, ÖNERİ(3), Rating(3), Rapor Tarihi, ONAY kararı(4)+Makam — onay alanları yalnız Komite rolünde aktif</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -4633,7 +4779,7 @@
     <row r="60">
       <c r="A60" s="15" t="inlineStr">
         <is>
-          <t>Overlay / İstisna Formu</t>
+          <t>Bulgu / Remediation Formu</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
@@ -4643,7 +4789,7 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Model*, Tür(5), Materyalite, Etki Yönü, Etki Tutarı, TFRS9 Aşaması, Senaryo, Gerekçe, Hesaplama, Kaldırma Kriteri, Onay Makamı, Bağımsız G.G.(4), Durum + Komite onay düğmeleri</t>
+          <t>Başlık*, Model, Kaynak(5), Önem(3→SLA), Remediation Durumu(6 aşama), Sorumlu, 2 tarih, Aksiyon Planı, Kanıt/Re-test — kapanış onay bloğu yalnız 2. hat</t>
         </is>
       </c>
       <c r="D60" s="15" t="inlineStr">
@@ -4657,7 +4803,7 @@
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>Guardrail Test Formu</t>
+          <t>Overlay / İstisna Formu</t>
         </is>
       </c>
       <c r="B61" s="16" t="inlineStr">
@@ -4667,7 +4813,7 @@
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Model(GenAI)*, Test Türü(7), Tarih, Sonuç(Geçti/Kaldı), Şiddet, Detay — 'Kaldı' otomatik bulgu</t>
+          <t>Model*, Tür(5), Materyalite, Etki Yönü, Etki Tutarı, TFRS9 Aşaması, Senaryo, Gerekçe, Hesaplama, Kaldırma Kriteri, Onay Makamı, Bağımsız G.G.(4), Durum + Komite onay düğmeleri</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -4681,7 +4827,7 @@
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t>Vendor Formu</t>
+          <t>Guardrail Test Formu</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
@@ -4691,7 +4837,7 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Tedarikçi, Şeffaflık(kara/gri/şeffaf), SLA, Çıkış Stratejisi, Kara-kutu Kısıtı, Due-Diligence(3), Son Gözden Geçirme</t>
+          <t>Model(GenAI)*, Test Türü(7), Tarih, Sonuç(Geçti/Kaldı), Şiddet, Detay — 'Kaldı' otomatik bulgu</t>
         </is>
       </c>
       <c r="D62" s="15" t="inlineStr">
@@ -4705,7 +4851,7 @@
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
         <is>
-          <t>Faz Formu (Model Journey)</t>
+          <t>Vendor Formu</t>
         </is>
       </c>
       <c r="B63" s="16" t="inlineStr">
@@ -4715,7 +4861,7 @@
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
-          <t>Faz başına R_Sxx_n alanları (dropdown/metin/sayı/tarih; * zorunlu) — 10 faz × 3-5 alan; kayıt ilerlemeyi besler</t>
+          <t>Tedarikçi, Şeffaflık(kara/gri/şeffaf), SLA, Çıkış Stratejisi, Kara-kutu Kısıtı, Due-Diligence(3), Son Gözden Geçirme</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -4726,8 +4872,32 @@
       <c r="E63" s="16" t="inlineStr"/>
       <c r="F63" s="16" t="inlineStr"/>
     </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>Faz Formu (Model Journey)</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>(özet)</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>Faz başına R_Sxx_n alanları (dropdown/metin/sayı/tarih; * zorunlu) — 10 faz × 3-5 alan; kayıt ilerlemeyi besler</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>karma</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr"/>
+      <c r="F64" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F63"/>
+  <autoFilter ref="A3:F64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4797,7 +4967,7 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>id (MDL-####), muid (HB-MDL-XXXXXXXXXXXX — benzersiz, DEĞİŞTİRİLEMEZ; oluşturmada atanır, düzenlemede korunur), karsilikEtkisi, ad, tip, sinif, modelTipi, kategori[], amac, amacDetay, metricProfile, aiml, genai, deterministik, duzenleyici, koken, tedarikci, sahipBirim, sahip, gelistirici, validator, metodoloji, algoritma, barindiran, durum, durumTalep, wf (mrm/komite/aktif/red), gelistirmeTarihi, prodTarihi, sonValidasyon, valFrekans, izlemeDurumu, upstream[], links{doc,monitor,repo,val}, kaynak, crit{M1-M5,K1-K7,B1,O1,duzenleyici,genai}, mat, kar, icsel, tier, derece, envanter{23 resmi alan,_auto}, vendor{}, phases[10], aimlEk{}, lifecyclePhase</t>
+          <t>id (MDL-####), muid (HB-MDL-XXXXXXXXXXXX — benzersiz, DEĞİŞTİRİLEMEZ; oluşturmada atanır, düzenlemede korunur), karsilikEtkisi, notaSurec (NOTA süreç kataloğu bağı), ihtiyacGerekce (zorunlu beyan gerekçesi), ad, tip, sinif, modelTipi, kategori[], amac, amacDetay, metricProfile, aiml, genai, deterministik, duzenleyici, koken, tedarikci, sahipBirim, sahip, gelistirici, validator, metodoloji, algoritma, barindiran, durum, durumTalep, wf (mrm/komite/aktif/red), gelistirmeTarihi, prodTarihi, sonValidasyon, valFrekans, izlemeDurumu, upstream[], links{doc,monitor,repo,val}, kaynak, crit{M1-M5,K1-K7,B1,O1,duzenleyici,genai}, mat, kar, icsel, tier, derece, envanter{23 resmi alan,_auto}, vendor{}, phases[10], aimlEk{}, lifecyclePhase</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Dokuman: tanitim Excel v1.3 — 'Dayanak & Atiflar' sayfasi (24 ozellik x birebir regülasyon alintisi: SR 11-7, SS1/23, OSFI E-23, EU AI Act, BDDK ISEDES, TFRS 9) + PMJ guncellemesi notu
</commit_message>
<xml_diff>
--- a/mrm-archer/MRM_Konsolu_Yazilim_Tanitim.xlsx
+++ b/mrm-archer/MRM_Konsolu_Yazilim_Tanitim.xlsx
@@ -8,24 +8,26 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak &amp; Kılavuz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menü Envanteri" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İşlemler (Use-Case)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formlar &amp; Alanlar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veri Modeli" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roller &amp; Yetki" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hesaplamalar" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bildirim &amp; E-posta" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Çıktılar &amp; Entegrasyon" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dayanak &amp; Atıflar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menü Envanteri" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İşlemler (Use-Case)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formlar &amp; Alanlar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veri Modeli" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roller &amp; Yetki" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hesaplamalar" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bildirim &amp; E-posta" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Çıktılar &amp; Entegrasyon" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Menü Envanteri'!$A$3:$F$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'İşlemler (Use-Case)'!$A$3:$H$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Formlar &amp; Alanlar'!$A$3:$F$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Veri Modeli'!$A$3:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roller &amp; Yetki'!$A$3:$F$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hesaplamalar'!$A$3:$C$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bildirim &amp; E-posta'!$A$14:$D$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Çıktılar &amp; Entegrasyon'!$A$3:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dayanak &amp; Atıflar'!$A$3:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Menü Envanteri'!$A$3:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'İşlemler (Use-Case)'!$A$3:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Formlar &amp; Alanlar'!$A$3:$F$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Veri Modeli'!$A$3:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Roller &amp; Yetki'!$A$3:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Hesaplamalar'!$A$3:$C$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Bildirim &amp; E-posta'!$A$14:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Çıktılar &amp; Entegrasyon'!$A$3:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -159,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +183,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -555,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -604,7 +609,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>v1.2 — bölümlü Yeni Model formu + upstream/downstream ilişki panelleri + NOTA süreci + zorunlu ihtiyaç gerekçesi</t>
+          <t>v1.3 — Dayanak &amp; Atıflar sayfası (birebir regülasyon alıntıları) + PMJ güncellemesi</t>
         </is>
       </c>
     </row>
@@ -808,41 +813,53 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Dayanak &amp; Atıflar</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>HER ÖZELLİĞİN regülatif dayanağı: kurum + doküman + bölüm + ORİJİNAL METİNDEKİ BİREBİR CÜMLE (yönetim sunumu için)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Özet sayılar (üretim betiğince sayılmıştır — statik doküman):</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Menü sayısı</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="n">
-        <v>25</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Tanımlı işlem sayısı</t>
+          <t>Menü sayısı</t>
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
+          <t>Tanımlı işlem sayısı</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>Form alanı sayısı</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n">
+      <c r="B30" s="12" t="n">
         <v>61</v>
       </c>
     </row>
@@ -856,10 +873,993 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E2001A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Çıktılar &amp; Entegrasyon Noktaları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Dışa/içe aktarımlar ve Archer entegrasyon karşılıkları</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Çıktı / Entegrasyon</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Nerede</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>İçerik / Kolonlar</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Not / Archer</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>XLSX Rapor (10 sheet)</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Üst çubuk düğmesi</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Özet(Board) · Model Envanteri · Validasyonlar · Validasyon Planı · Bulgular · Overlay-PMA · Guardrail · Son Metrikler · BDDK Kanıt · Denetim İzi</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Saf JS xlsx yazıcı (harici kütüphane yok); Archer Reporting/mail-merge karşılığı</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Envanter CSV dışa</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Model Envanteri</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Model ID, MUID, Model Adı, İş Birimi, Sınıf, Model Tipi, Kategori, Durum, Metrik Çerçevesi, Düzenleyici, AI/ML, Genel Kritiklik, Son Validasyon, Tier, İçsel Risk, Kaynak</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Şablon olarak da kullanılır</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>CSV toplu içe aktarma</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Model Envanteri</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Başlık eşleştirme esnek (TR); zorunlu: Model Adı; Tier/metrik/takvim otomatik; kayıtlar onay akışına girer</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Archer Data Import / Data Feed Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>BDDK kanıt CSV/PDF</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>BDDK / İSEDES</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Model, Tier, İSEDES bağı, validasyon güncelliği, açık bulgu, overlay</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>JSON yedek/geri yükle</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Hakkında</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Tüm state (models, validations, findings, metrics, pmas, changes, guardrails, audit, tmrHistory)</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Taşınabilirlik/test</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Günlük özet e-postası</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Bildirim</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Özet metin + mailto: + panoya kopyala</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Notifications digest</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Veri Feed / API (simülasyon)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Veri Feed</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Feed tanımları ve örnek payload görünümü</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Data Feed Manager / REST API</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Board raporu (yazdır)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Risk Panosu</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>window.print ile PDF</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E2001A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Dayanak &amp; Atıflar — Özellik → Regülatif Kaynak → Orijinal Cümle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Alıntılar kaynak metinlerden BİREBİR alınmıştır (doğrulama: resmi PDF/metinler). Kısaltmalar: SR 11-7 = Fed SR 11-7 / OCC 2011-12 (04.04.2011) · SS1/23 = Bank of England PRA SS1/23 (May 2023) · E-23 = OSFI Guideline E-23 (2027) · AI Act = Regulation (EU) 2024/1689 · İSEDES Yön. = BDDK, RG 11.07.2014-29057 · TFRS 9 = IFRS 9 (KGK çevirisi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Uygulamadaki Özellik</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Kaynak Kurum</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Doküman · Bölüm</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>ORİJİNAL METİNDEKİ CÜMLE (birebir alıntı)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Neden / Bizim Uygulamamız</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>MRM'in ayrı bir risk disiplini olarak kurulması (tüm konsol)</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Bank of England (PRA)</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>SS1/23, §1.4</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>The PRA's desired outcome is that firms take a strategic approach to MRM as a risk discipline in its own right.</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Model riskini kredi/piyasa riski gibi başlı başına bir disiplin olarak yöneten ayrı bir konsol kurduk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Model tanımı &amp; kapsam (tüm model/algoritmalar envanterde)</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Overview of Model Risk Management'</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>...the term model refers to a quantitative method, system, or approach that applies statistical, economic, financial, or mathematical theories, techniques, and assumptions to process input data into quantitative estimates.</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Bu tanım Hakkında sayfasındaki 'model karar ağacı'nın ve envanter kapsamının (istatistiksel/ekonometrik/AI-ML/kural) temelidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Kurum-geneli Model Envanteri ekranı</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Model Inventory'</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Banks should maintain a comprehensive set of information for models implemented for use, under development for implementation, or recently retired.</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Envanter tüm durumları (Geliştirme→Emekli) kapsar; birim×sınıf matrisi banka genelini gösterir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Envanter alan seti + MUID (değiştirilemez kimlik) + 'evergreen' güncellik</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>OSFI (Kanada)</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Guideline E-23 (2027), §C.1</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>An institution's model inventory should be... accurate, evergreen, and subject to robust controls...</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Benzersiz-değiştirilemez MUID, denetim izi ve onay akışı envanterin 'doğru, güncel ve kontrollü' tutulmasının sistemsel karşılığıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Envanterde bağımlılıklar + Bağımlılık &amp; Etki sayfası</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Bank of England (PRA)</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>SS1/23, Principle 1.2</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>A comprehensive model inventory should be maintained to enable firms to: identify the sources of model risk; provide the management information needed for reporting model risk; and help to identify model inter-dependencies.</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Upstream/downstream ilişki panelleri ve ağ grafiği 'model inter-dependencies' beklentisinin doğrudan uygulamasıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Kritiklik Değerlendirmesi → Tier 1-3/Sınıf (risk-bazlı tiering)</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Bank of England (PRA)</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>SS1/23, Principle 1.3</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Risk-based model tiering should be used to prioritise validation activities and other risk controls through the model lifecycle, and to identify and classify those models that pose most risk to a firm's business activities, and/or firm safety and soundness.</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Materyalite×Karmaşıklık skoru ile tier ataması ve tier'a göre validasyon frekansı/eşikler bu prensipten türetildi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Bağımsız Validasyon + ÖNERİ ≠ ONAY (etkin sorgulama)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Overview'</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>A guiding principle for managing model risk is 'effective challenge' of models, that is, critical analysis by objective, informed parties who can identify model limitations and assumptions and produce appropriate changes.</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Validasyon test kataloğu + etkin sorgulama notları alanı bu ilkeye dayanır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Validasyon bağımsızlığı (rol ayrımı, alan kilitleri)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Model Validation'</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Validation involves a degree of independence from model development and use. Generally, validation should be done by people who are not responsible for development or use and do not have a stake in whether a model is determined to be valid.</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Öneri/rating alanları yalnız bağımsız validasyon rolünde; onay ayrı makamda (görevler ayrılığı).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Validasyon Planı — yıllık/risk-bazlı takvim + gecikme uyarıları</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Model Validation'</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Banks should conduct a periodic review—at least annually but more frequently if warranted—of each model to determine whether it is working as intended and if the existing validation activities are sufficient.</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>12 aylık takvim, Tier-bazlı frekans (T1 yıllık) ve 'Gecikmiş' uyarıları bu cümlenin operasyonelleştirilmesidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>İzleme &amp; Metrikler (PSI/AUC eşikleri, drift → aksiyon)</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Ongoing Monitoring'</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Ongoing monitoring is essential to evaluate whether changes in products, exposures, activities, clients, or market conditions necessitate adjustment, redevelopment, or replacement of the model and to verify that any extension of the model beyond its original scope is valid.</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Metrik zaman serileri, tier-bazlı eşikler ve eşik aşımı→bulgu otomasyonu buradan gelir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Geriye dönük test (backtesting) zorunluluğu</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>BDDK</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>İSEDES Yönetmeliği, md.42/6</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Risk ölçüm yöntemi veya modelinin doğruluğu ve güvenilirliği, gerçekleşen sonuçlar kullanılarak geriye dönük testler yoluyla tespit edilir.</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Validasyon test kataloğundaki backtesting maddesi ve izleme serileri bu hükmün karşılığıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Validasyon tanımı (BDDK uyumu)</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>BDDK</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>İSEDES Yönetmeliği, md.3/1(ll)</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Validasyon: Metodoloji kapsamında kullanılan modellerin gerçekleşmeleri hangi oranda temsil ettiğini kesinlik, doğruluk ve tutarlılık ölçüleri kullanılarak belirlenmesi ve metodolojinin diğer unsurlarının sağlamlığının değerlendirilmesini [ifade eder].</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Validasyon modülündeki test seti (kesinlik/doğruluk/tutarlılık) bu tanımla hizalıdır; BDDK/İSEDES Kanıt sayfası bu bağı raporlar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Toplam Model Riski Endeksi (toplulaştırılmış risk)</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Overview'</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Banks should consider risk from individual models and in the aggregate. Aggregate model risk is affected by interaction and dependencies among models; reliance on common assumptions, data, or methodologies; and any other factors that could adversely affect several models and their outputs at the same time.</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>0-100 TMR endeksi + bağımlılık ağı 'aggregate model risk' beklentisinin panosudur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Risk İştahı eşikleri (board göstergesi)</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Bank of England (PRA)</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>SS1/23, Principle 2</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Firms should have strong governance oversight with a board that promotes an MRM culture from the top through setting clear model risk appetite.</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Amber/kırmızı iştah eşikleri ve board tek-sayfa özeti bu prensibe dayanır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Board/üst yönetim yönetişimi</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Governance'</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Model risk governance is provided at the highest level by the board of directors and senior management when they establish a bank-wide approach to model risk management.</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Risk Panosu &amp; Board ekranı + öz-değerlendirme/attestasyon bu çerçeveyi sunar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>TFRS9 BKZ Overlay (PMA) yönetişimi + bağımsız gözden geçirme</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Bank of England (PRA)</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>SS1/23, Principle 5</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Firms should have established policies and procedures for the use of model risk mitigants when models are under-performing, and should have procedures for the independent review of post-model adjustments.</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Overlay kayıtları (etki/aşama/senaryo), Komite onayı ve bağımsız G.G. alanı P5'in birebir uygulamasıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Overlay'in muhasebe dayanağı (ileriye dönük bilgi)</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>KGK / IASB</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>TFRS 9 / IFRS 9, prg. 5.5.17(c)</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>...reasonable and supportable information that is available without undue cost or effort at the reporting date about past events, current conditions and forecasts of future economic conditions.</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>Makro belirsizlikte ECL üzerine overlay gereği bu paragraftan doğar; kayıtta senaryo bağı alanı bulunur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Kullanım istisnası / PMA eskalasyonu</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Bank of England (PRA)</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>SS1/23, Principle 5.3</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Exceptions for model use should be temporary, should be subject to post-model adjustments (PMAs), should be reported to and supported by stakeholders and senior management.</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>İstisna kayıtları geçicilik + kaldırma kriteri + onay makamı alanlarıyla modellenmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Bulgu remediation + kısıtlı kullanım</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Model Validation'</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>If significant deficiencies are noted as a result of the validation process, use of the model should not be allowed or should be permitted only under very tight constraints until those issues are resolved.</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Bulgu yaşam döngüsü (kanıt+2.hat kapanış onayı) ve 'Kısıtlı/Askıda' durumu bu hükmü uygular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Model Değişiklik → materyal değişiklikte revalidasyon</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Model Validation'</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Material changes to models should also be subject to validation.</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Değişiklik kaydındaki materyalite alanı revalidasyon tetiğini işaretler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Vendor &amp; 3. taraf model yönetişimi</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Third-Party Products'</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Vendor products should nevertheless be incorporated into a bank's broader model risk management framework following the same principles as applied to in-house models, although the process may be somewhat modified.</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Vendor ekranı (due-diligence, SLA, çıkış stratejisi, kara-kutu kısıtı) bu cümlenin uygulamasıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Model Journey — 10 fazlı yaşam döngüsü</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>OSFI (Kanada)</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Guideline E-23 (2027), §A tanımlar</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Model lifecycle components are model design (including model rationale, data, and development), model review, model deployment, model monitoring, and model decommission.</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>10 fazlı stepper + faz form motoru yaşam döngüsünün uçtan uca yönetimidir; E-23 Outcome: 'Model risk is managed using a risk-based approach.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>EU AI Act uyum izleyici (yüksek riskli AI)</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Avrupa Birliği</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>AI Act (2024/1689), Madde 9(1)-(2)</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>A risk management system shall be established, implemented, documented and maintained in relation to high-risk AI systems. / The risk management system shall be understood as a continuous iterative process planned and run throughout the entire lifecycle of a high-risk AI system, requiring regular systematic review and updating.</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Madde-bazlı uyum izleyici ve boşluk→bulgu otomasyonu bu yükümlülüğü canlandırır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>GenAI guardrail / red-team logu (Generative &amp; Agentic AI)</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Avrupa Birliği</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>AI Act (2024/1689), Madde 15(1) ve 15(5)</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>High-risk AI systems shall be designed and developed in such a way that they achieve an appropriate level of accuracy, robustness, and cybersecurity... / High-risk AI systems shall be resilient against attempts by unauthorised third parties to alter their use, outputs or performance by exploiting system vulnerabilities.</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Prompt injection/jailbreak/red-team test kayıtları ve başarısızlıkta otomatik bulgu, 'robustness/resilience' hükümlerinin test kanıtıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Denetim izi + işlem içeriği (alan bazlı önce→sonra)</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>ABD Fed / OCC</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>SR 11-7, 'Documentation'</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Without adequate documentation, model risk assessment and management will be ineffective.</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>Değişmez denetim izi + tıklanır alan-bazlı değişiklik içeriği (Archer History Log) bu ilkeden doğar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Kaynak erişimleri: SR 11-7 federalreserve.gov/boarddocs/srletters/2011/sr1107a1.pdf · SS1/23 bankofengland.co.uk (PS6/23 eki) · OSFI E-23 osfi-bsif.gc.ca · AI Act eur-lex.europa.eu (2024/1689) · İSEDES Yön. RG 11.07.2014-29057 · TFRS 9 kgk.gov.tr. Alıntılar bu resmi metinlerden birebir aktarılmıştır; köşeli parantez [ ] editoryal tamamlamadır, üç nokta (…) atlanan bölümü gösterir.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:E28"/>
+  <mergeCells count="1">
+    <mergeCell ref="A30:E30"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00004A93"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1726,10 +2726,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00004A93"/>
+    <tabColor rgb="00E2001A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3152,10 +4152,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00E2001A"/>
+    <tabColor rgb="00004A93"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -4902,10 +5902,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00004A93"/>
+    <tabColor rgb="00E2001A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -5202,10 +6202,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00E2001A"/>
+    <tabColor rgb="00004A93"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -5811,7 +6811,7 @@
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Özel kurallar: Varsayılan rol 1. Hat. ÖNERİ ≠ ONAY (validasyon bağımsızlığı). 3. Hat için tüm primary düğmeler + beyan girişi CSS ile kilitlenir; ayrıca işlem fonksiyonları (guardWrite/roleGuard/roGuard) programatik engeller. Onay adımları görevler ayrılığıyla zorlanır.</t>
         </is>
@@ -5826,10 +6826,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00004A93"/>
+    <tabColor rgb="00E2001A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -6218,10 +7218,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00E2001A"/>
+    <tabColor rgb="00004A93"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -6615,7 +7615,7 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Talep: Bu kurallar Archer Notifications + Advanced Workflow notification şablonları ve scheduled report/digest ile e-posta olarak uygulanacaktır. Uygulamada giden kutusu simülasyonu ve günlük özet önizlemesi (mailto) mevcuttur.</t>
         </is>
@@ -6628,238 +7628,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00004A93"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>Çıktılar &amp; Entegrasyon Noktaları</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>Dışa/içe aktarımlar ve Archer entegrasyon karşılıkları</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Çıktı / Entegrasyon</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Nerede</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>İçerik / Kolonlar</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Not / Archer</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>XLSX Rapor (10 sheet)</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Üst çubuk düğmesi</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Özet(Board) · Model Envanteri · Validasyonlar · Validasyon Planı · Bulgular · Overlay-PMA · Guardrail · Son Metrikler · BDDK Kanıt · Denetim İzi</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>Saf JS xlsx yazıcı (harici kütüphane yok); Archer Reporting/mail-merge karşılığı</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Envanter CSV dışa</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Model Envanteri</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Model ID, MUID, Model Adı, İş Birimi, Sınıf, Model Tipi, Kategori, Durum, Metrik Çerçevesi, Düzenleyici, AI/ML, Genel Kritiklik, Son Validasyon, Tier, İçsel Risk, Kaynak</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>Şablon olarak da kullanılır</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>CSV toplu içe aktarma</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Model Envanteri</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Başlık eşleştirme esnek (TR); zorunlu: Model Adı; Tier/metrik/takvim otomatik; kayıtlar onay akışına girer</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Archer Data Import / Data Feed Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>BDDK kanıt CSV/PDF</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>BDDK / İSEDES</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>Model, Tier, İSEDES bağı, validasyon güncelliği, açık bulgu, overlay</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>JSON yedek/geri yükle</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Hakkında</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Tüm state (models, validations, findings, metrics, pmas, changes, guardrails, audit, tmrHistory)</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>Taşınabilirlik/test</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Günlük özet e-postası</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Bildirim</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Özet metin + mailto: + panoya kopyala</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Notifications digest</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>Veri Feed / API (simülasyon)</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Veri Feed</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Feed tanımları ve örnek payload görünümü</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>Data Feed Manager / REST API</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Board raporu (yazdır)</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Risk Panosu</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>window.print ile PDF</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:D11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>